<commit_message>
chore: sync all project files and logs for latest working version
</commit_message>
<xml_diff>
--- a/logs/Forward Testing Trade History.xlsx
+++ b/logs/Forward Testing Trade History.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1660,6 +1660,240 @@
         <v>103479</v>
       </c>
     </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07 09:20:02</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59900PE</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>454.45</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07 09:22:15</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>442.75</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>431.73</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>522.62</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>431.73</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>-409.5</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>-459.5</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>15905.75</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>89.25</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>-728</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>-4.58</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="V16" s="2" t="n">
+        <v>103069.5</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07 09:52:01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59900PE</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>454.45</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07 10:15:09</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>431.25</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>431.73</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>522.62</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>431.73</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>-812</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>-862</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>15905.75</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>948.5</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>-812</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="V17" s="2" t="n">
+        <v>102667</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08 09:20:02</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59800PE</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>433.6</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08 09:34:41</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>410.5</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>411.92</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>498.64</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>411.92</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>-808.5</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>-858.5</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>15176</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>-808.5</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="V18" s="2" t="n">
+        <v>102670.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: archive log after session for complete session logs; ensure archiving works with both direct and start_strategy.py runs
</commit_message>
<xml_diff>
--- a/logs/Forward Testing Trade History.xlsx
+++ b/logs/Forward Testing Trade History.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1894,6 +1894,708 @@
         <v>102670.5</v>
       </c>
     </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09 09:20:03</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59500PE</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>403.95</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09 10:28:02</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>382.1</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>383.75</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>464.54</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>383.75</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>-764.75</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>-814.75</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>14138.25</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>-5.41</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>1891.75</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>-764.75</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>-5.41</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="V19" s="2" t="n">
+        <v>102714.25</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12 09:20:08</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59000PE</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>416.95</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12 09:31:26</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>394.7</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>396.1</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>479.49</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>396.1</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>-778.75</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>-828.75</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>14593.25</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>-5.34</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>549.5</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>-778.75</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>-5.34</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="V20" s="2" t="n">
+        <v>102700.25</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12 09:36:02</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59000PE</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>416.95</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12 10:27:45</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>366.6</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>375.26</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>458.65</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>375.26</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>-1762.25</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>-1812.25</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>14593.25</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>-12.08</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>211.75</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>-1762.25</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>-12.08</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="V21" s="2" t="n">
+        <v>101716.75</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13 09:20:02</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59600PE</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>457.15</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13 09:43:09</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>503</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>411.44</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>502.87</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>411.44</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>1604.75</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>1554.75</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>16000.25</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>1604.75</v>
+      </c>
+      <c r="R22" s="2" t="n">
+        <v>-518</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>-3.24</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="V22" s="2" t="n">
+        <v>105083.75</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 09:20:02</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59600CE</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>607.1</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 09:23:23</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>573.7</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>576.75</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>637.46</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>576.75</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>-1169</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>-1219</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>21248.5</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>775.25</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>-1169</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="V23" s="2" t="n">
+        <v>102310</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 09:37:08</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59600CE</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>607.1</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 09:40:19</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>574.5</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>576.75</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>637.46</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>576.75</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>-1141</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>-1191</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>21248.5</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>-5.37</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>-49</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>-1141</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>-5.37</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="V24" s="2" t="n">
+        <v>102338</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 09:20:02</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59800CE</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>522.7</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 09:43:33</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>550.05</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>496.56</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>548.84</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>496.56</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>957.25</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>907.25</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>18294.5</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>957.25</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>-890.75</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>-4.87</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="V25" s="2" t="n">
+        <v>104436.25</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 10:35:40</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59800CE</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>522.7</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 10:35:51</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>743.2</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>496.56</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>548.84</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>496.56</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>7717.5</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>7667.5</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>18294.5</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>42.18</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>7717.5</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>7717.5</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>42.18</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>42.18</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="V26" s="2" t="n">
+        <v>111196.5</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-19 09:20:02</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59800PE</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>380.05</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-19 09:58:21</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>419.2</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>342.05</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>418.06</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>342.05</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>1370.25</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>1320.25</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>13301.75</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>1370.25</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>-575.75</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>-4.33</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="V27" s="2" t="n">
+        <v>101370.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Backup: commit all current project files before analysis script addition
</commit_message>
<xml_diff>
--- a/logs/Forward Testing Trade History.xlsx
+++ b/logs/Forward Testing Trade History.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -440,7 +440,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
@@ -2596,6 +2596,2346 @@
         <v>101370.25</v>
       </c>
     </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20 09:20:02</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59800PE</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>375.1</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20 09:54:02</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>414.55</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>337.59</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>412.61</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>337.59</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>1380.75</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>1330.75</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>13128.5</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>1380.75</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>-341.25</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="V28" s="2" t="n">
+        <v>101380.75</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21 09:20:03</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59100PE</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>261.05</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21 09:59:06</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>287.4</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>234.95</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>287.16</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>234.95</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>922.25</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>872.25</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>9136.75</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>922.25</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>-537.25</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>-5.88</v>
+      </c>
+      <c r="U29" s="2" t="n">
+        <v>13.07</v>
+      </c>
+      <c r="V29" s="2" t="n">
+        <v>100922.25</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22 09:20:02</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59300CE</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>400.1</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22 09:21:05</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>360.09</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>440.11</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>360.09</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>1746.5</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>1696.5</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>14003.5</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>1746.5</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>234.5</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="U30" s="2" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="V30" s="2" t="n">
+        <v>101746.5</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23 09:35:31</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59100PE</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>264.1</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23 09:45:22</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>294.15</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>237.69</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>290.51</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>237.69</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>1051.75</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>1001.75</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>9243.5</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>1051.75</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>-393.75</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="T31" s="2" t="n">
+        <v>-4.26</v>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>13.68</v>
+      </c>
+      <c r="V31" s="2" t="n">
+        <v>99912.25</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23 09:35:31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN59100PE</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>264.1</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23 09:45:22</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>294.15</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>237.69</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>290.51</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>237.69</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>1051.75</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>1001.75</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>9243.5</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>1051.75</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>-393.75</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="T32" s="2" t="n">
+        <v>-4.26</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>13.68</v>
+      </c>
+      <c r="V32" s="2" t="n">
+        <v>99912.25</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27 09:20:02</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN58300PE</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>242.95</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27 09:21:58</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>267.25</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>968.5</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>8503.25</v>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="R33" s="2" t="n">
+        <v>-442.75</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>-5.21</v>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="V33" s="2" t="n">
+        <v>100880.75</v>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27 09:20:02</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26JAN58300PE</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>242.95</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27 09:21:59</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>267.25</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>968.5</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>8503.25</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>-442.75</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="T34" s="2" t="n">
+        <v>-5.21</v>
+      </c>
+      <c r="U34" s="2" t="n">
+        <v>15.97</v>
+      </c>
+      <c r="V34" s="2" t="n">
+        <v>100880.75</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28 09:20:02</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB59600CE</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>1110.75</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28 11:42:40</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>1053.05</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>1055.21</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>1166.29</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>1055.21</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>-2019.5</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>-2069.5</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>38876.25</v>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>-5.19</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>864.5</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>-2019.5</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="T35" s="2" t="n">
+        <v>-5.19</v>
+      </c>
+      <c r="U35" s="2" t="n">
+        <v>13.82</v>
+      </c>
+      <c r="V35" s="2" t="n">
+        <v>98811.25</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 09:20:02</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB59500CE</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>1055.55</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 09:50:22</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>1108.9</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>1002.77</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>1108.33</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>1002.77</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>1867.25</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>1817.25</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>36944.25</v>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>1867.25</v>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>-787.5</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="T36" s="2" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="U36" s="2" t="n">
+        <v>13.82</v>
+      </c>
+      <c r="V36" s="2" t="n">
+        <v>100628.5</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30 09:20:02</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB59500PE</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>685.85</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30 09:23:04</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>720.9</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>651.5599999999999</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>720.14</v>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>651.5599999999999</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>1226.75</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>1176.75</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>24004.75</v>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>1226.75</v>
+      </c>
+      <c r="R37" s="2" t="n">
+        <v>281.75</v>
+      </c>
+      <c r="S37" s="2" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="T37" s="2" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="U37" s="2" t="n">
+        <v>13.78</v>
+      </c>
+      <c r="V37" s="2" t="n">
+        <v>101805.25</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01 09:40:04</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB59500PE</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>755.1</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01 09:51:06</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>717.35</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>792.86</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>717.35</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>-1928.5</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>-1978.5</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>26428.5</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>-267.75</v>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>-1928.5</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="T38" s="2" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="U38" s="2" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="V38" s="2" t="n">
+        <v>99826.75</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:20:02</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB58300CE</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>1109.9</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:23:02</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>1165.6</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>1054.4</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>1165.39</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>1054.4</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>1949.5</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>1899.5</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>38846.5</v>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>1949.5</v>
+      </c>
+      <c r="R39" s="2" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="U39" s="2" t="n">
+        <v>15.26</v>
+      </c>
+      <c r="V39" s="2" t="n">
+        <v>101726.25</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:20:02</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60000PE</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>770.05</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:20:51</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>726.7</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>731.55</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>808.55</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>731.55</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>-1517.25</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>-1567.25</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>26951.75</v>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>-5.63</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>295.75</v>
+      </c>
+      <c r="R40" s="2" t="n">
+        <v>-1517.25</v>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="T40" s="2" t="n">
+        <v>-5.63</v>
+      </c>
+      <c r="U40" s="2" t="n">
+        <v>14.69</v>
+      </c>
+      <c r="V40" s="2" t="n">
+        <v>100159</v>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-04 09:20:02</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60200CE</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>786.05</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-04 09:45:18</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>826</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>746.75</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>825.35</v>
+      </c>
+      <c r="J41" s="2" t="n">
+        <v>746.75</v>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>1398.25</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>1348.25</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>27511.75</v>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>1398.25</v>
+      </c>
+      <c r="R41" s="2" t="n">
+        <v>-560</v>
+      </c>
+      <c r="S41" s="2" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="T41" s="2" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="U41" s="2" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="V41" s="2" t="n">
+        <v>101507.25</v>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05 09:20:02</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60200PE</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>629.05</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05 10:21:57</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>592.9</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>597.6</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>660.5</v>
+      </c>
+      <c r="J42" s="2" t="n">
+        <v>597.6</v>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>-1265.25</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>-1315.25</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>22016.75</v>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>-5.75</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>665</v>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>-1265.25</v>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="T42" s="2" t="n">
+        <v>-5.75</v>
+      </c>
+      <c r="U42" s="2" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="V42" s="2" t="n">
+        <v>100192</v>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-06 09:20:02</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60100CE</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>708.1</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-06 09:38:14</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>671.9</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>672.6900000000001</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>743.51</v>
+      </c>
+      <c r="J43" s="2" t="n">
+        <v>672.6900000000001</v>
+      </c>
+      <c r="K43" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>-1267</v>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>-1317</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>24783.5</v>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>717.5</v>
+      </c>
+      <c r="R43" s="2" t="n">
+        <v>-1267</v>
+      </c>
+      <c r="S43" s="2" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="T43" s="2" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="U43" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="V43" s="2" t="n">
+        <v>98875</v>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 09:20:02</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60900CE</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>481.65</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 10:28:30</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>432.85</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>433.49</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>529.8200000000001</v>
+      </c>
+      <c r="J44" s="2" t="n">
+        <v>433.49</v>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M44" s="2" t="n">
+        <v>-1708</v>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>-1758</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>16857.75</v>
+      </c>
+      <c r="P44" s="2" t="n">
+        <v>-10.13</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>665</v>
+      </c>
+      <c r="R44" s="2" t="n">
+        <v>-1708</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="T44" s="2" t="n">
+        <v>-10.13</v>
+      </c>
+      <c r="U44" s="2" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="V44" s="2" t="n">
+        <v>97117</v>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10 09:20:02</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60800CE</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>512.25</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:37:21</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>485.6</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>486.64</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>537.86</v>
+      </c>
+      <c r="J45" s="2" t="n">
+        <v>486.64</v>
+      </c>
+      <c r="K45" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M45" s="2" t="n">
+        <v>-932.75</v>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>-982.75</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>17928.75</v>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>516.25</v>
+      </c>
+      <c r="R45" s="2" t="n">
+        <v>-932.75</v>
+      </c>
+      <c r="S45" s="2" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="T45" s="2" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="U45" s="2" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="V45" s="2" t="n">
+        <v>96134.25</v>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11 09:20:02</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60500PE</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>393.45</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11 09:40:05</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>435.1</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>354.11</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>432.8</v>
+      </c>
+      <c r="J46" s="2" t="n">
+        <v>354.11</v>
+      </c>
+      <c r="K46" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L46" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M46" s="2" t="n">
+        <v>1457.75</v>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>1407.75</v>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>13770.75</v>
+      </c>
+      <c r="P46" s="2" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>1457.75</v>
+      </c>
+      <c r="R46" s="2" t="n">
+        <v>-117.25</v>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="T46" s="2" t="n">
+        <v>-0.85</v>
+      </c>
+      <c r="U46" s="2" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="V46" s="2" t="n">
+        <v>97542</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12 09:20:02</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60800CE</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>455.65</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12 10:14:07</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>410.09</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>501.22</v>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>410.09</v>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>1692.25</v>
+      </c>
+      <c r="N47" s="2" t="n">
+        <v>1642.25</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>15947.75</v>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>1692.25</v>
+      </c>
+      <c r="R47" s="2" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="S47" s="2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="T47" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="U47" s="2" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="V47" s="2" t="n">
+        <v>99184.25</v>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13 09:20:02</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB60400PE</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>368.25</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13 10:15:05</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>405.15</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>331.43</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>405.08</v>
+      </c>
+      <c r="J48" s="2" t="n">
+        <v>331.43</v>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L48" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M48" s="2" t="n">
+        <v>1291.5</v>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>1241.5</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>12888.75</v>
+      </c>
+      <c r="P48" s="2" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>1291.5</v>
+      </c>
+      <c r="R48" s="2" t="n">
+        <v>-390.25</v>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="T48" s="2" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="U48" s="2" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="V48" s="2" t="n">
+        <v>100425.75</v>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:20:02</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB61300CE</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>308.2</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:56:04</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>273.9</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>277.38</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>339.02</v>
+      </c>
+      <c r="J49" s="2" t="n">
+        <v>277.38</v>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M49" s="2" t="n">
+        <v>-1200.5</v>
+      </c>
+      <c r="N49" s="2" t="n">
+        <v>-1250.5</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>10787</v>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>-11.13</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>1036</v>
+      </c>
+      <c r="R49" s="2" t="n">
+        <v>-1200.5</v>
+      </c>
+      <c r="S49" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="T49" s="2" t="n">
+        <v>-11.13</v>
+      </c>
+      <c r="U49" s="2" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="V49" s="2" t="n">
+        <v>99175.25</v>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23 09:26:35</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26FEB61300CE</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>297.1</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23 09:26:46</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>351.3</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>267.39</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>326.81</v>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>267.39</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M50" s="2" t="n">
+        <v>1897</v>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>1847</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>10398.5</v>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>1897</v>
+      </c>
+      <c r="R50" s="2" t="n">
+        <v>1897</v>
+      </c>
+      <c r="S50" s="2" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="T50" s="2" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="U50" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="V50" s="2" t="n">
+        <v>101022.25</v>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:20:02</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR61300CE</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>1044.35</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:53:41</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>986.3</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>992.13</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>1096.57</v>
+      </c>
+      <c r="J51" s="2" t="n">
+        <v>992.13</v>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>-2031.75</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>-2081.75</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>36552.25</v>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>-5.56</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>582.75</v>
+      </c>
+      <c r="R51" s="2" t="n">
+        <v>-2031.75</v>
+      </c>
+      <c r="S51" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="T51" s="2" t="n">
+        <v>-5.56</v>
+      </c>
+      <c r="U51" s="2" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="V51" s="2" t="n">
+        <v>98940.5</v>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26 09:20:02</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR61100PE</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>698.9</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26 09:36:51</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>662</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>663.95</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>733.85</v>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>663.95</v>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M52" s="2" t="n">
+        <v>-1291.5</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>-1341.5</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>24461.5</v>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>213.5</v>
+      </c>
+      <c r="R52" s="2" t="n">
+        <v>-1291.5</v>
+      </c>
+      <c r="S52" s="2" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="T52" s="2" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="U52" s="2" t="n">
+        <v>13.19</v>
+      </c>
+      <c r="V52" s="2" t="n">
+        <v>97599</v>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27 09:20:02</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR60900PE</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>675.1</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27 09:36:32</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>709</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>641.35</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>708.86</v>
+      </c>
+      <c r="J53" s="2" t="n">
+        <v>641.35</v>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L53" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M53" s="2" t="n">
+        <v>1186.5</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>1136.5</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>23628.5</v>
+      </c>
+      <c r="P53" s="2" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>1186.5</v>
+      </c>
+      <c r="R53" s="2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="S53" s="2" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="T53" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="U53" s="2" t="n">
+        <v>13.48</v>
+      </c>
+      <c r="V53" s="2" t="n">
+        <v>98735.5</v>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:24:21</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR60100CE</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>1132.9</v>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:28:55</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>1193</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>1076.25</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>1189.54</v>
+      </c>
+      <c r="J54" s="2" t="n">
+        <v>1076.25</v>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>2103.5</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>2053.5</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>39651.5</v>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>2103.5</v>
+      </c>
+      <c r="R54" s="2" t="n">
+        <v>-441</v>
+      </c>
+      <c r="S54" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="T54" s="2" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="U54" s="2" t="n">
+        <v>16.11</v>
+      </c>
+      <c r="V54" s="2" t="n">
+        <v>100789</v>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05 09:20:02</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR58800PE</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>990.05</v>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05 14:24:53</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>901.25</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>940.55</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>1039.55</v>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>940.55</v>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>-3108</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>-3158</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>34651.75</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>-8.970000000000001</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>995.75</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>-3108</v>
+      </c>
+      <c r="S55" s="2" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="T55" s="2" t="n">
+        <v>-8.970000000000001</v>
+      </c>
+      <c r="U55" s="2" t="n">
+        <v>18.66</v>
+      </c>
+      <c r="V55" s="2" t="n">
+        <v>97631</v>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06 09:20:02</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR58500PE</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>853.1</v>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06 09:35:06</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>899</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>810.4400000000001</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>895.76</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>810.4400000000001</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>1606.5</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>1556.5</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>29858.5</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>1606.5</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>-539</v>
+      </c>
+      <c r="S56" s="2" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="T56" s="2" t="n">
+        <v>-1.81</v>
+      </c>
+      <c r="U56" s="2" t="n">
+        <v>18.36</v>
+      </c>
+      <c r="V56" s="2" t="n">
+        <v>99187.5</v>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09 10:43:40</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR55500PE</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>1340.1</v>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09 10:43:50</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>1437.3</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>1273.09</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>1407.11</v>
+      </c>
+      <c r="J57" s="2" t="n">
+        <v>1273.09</v>
+      </c>
+      <c r="K57" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L57" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M57" s="2" t="n">
+        <v>3402</v>
+      </c>
+      <c r="N57" s="2" t="n">
+        <v>3352</v>
+      </c>
+      <c r="O57" s="2" t="n">
+        <v>46903.5</v>
+      </c>
+      <c r="P57" s="2" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>3402</v>
+      </c>
+      <c r="R57" s="2" t="n">
+        <v>3402</v>
+      </c>
+      <c r="S57" s="2" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="T57" s="2" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="U57" s="2" t="n">
+        <v>24.22</v>
+      </c>
+      <c r="V57" s="2" t="n">
+        <v>102539.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
SEBI/Fyers API compliance: All regulatory updates complete as of April 2026
</commit_message>
<xml_diff>
--- a/logs/Forward Testing Trade History.xlsx
+++ b/logs/Forward Testing Trade History.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V57"/>
+  <dimension ref="A1:V70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4936,6 +4936,1020 @@
         <v>102539.5</v>
       </c>
     </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12 09:20:02</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR55100CE</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1271.95</v>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12 09:51:50</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>1365</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>1182.91</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>1360.99</v>
+      </c>
+      <c r="J58" s="2" t="n">
+        <v>1182.91</v>
+      </c>
+      <c r="K58" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L58" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M58" s="2" t="n">
+        <v>3256.75</v>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>3206.75</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>44518.25</v>
+      </c>
+      <c r="P58" s="2" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>3256.75</v>
+      </c>
+      <c r="R58" s="2" t="n">
+        <v>-145.25</v>
+      </c>
+      <c r="S58" s="2" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="T58" s="2" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="U58" s="2" t="n">
+        <v>22.11</v>
+      </c>
+      <c r="V58" s="2" t="n">
+        <v>105746.25</v>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12 14:45:31</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR55100CE</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>1271.95</v>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12 14:45:41</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>1385.8</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>1182.91</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>1360.99</v>
+      </c>
+      <c r="J59" s="2" t="n">
+        <v>1182.91</v>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M59" s="2" t="n">
+        <v>3984.75</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>3934.75</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>44518.25</v>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>3984.75</v>
+      </c>
+      <c r="R59" s="2" t="n">
+        <v>3984.75</v>
+      </c>
+      <c r="S59" s="2" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="T59" s="2" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="U59" s="2" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="V59" s="2" t="n">
+        <v>109681</v>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13 09:20:02</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR54500PE</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>1077.7</v>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13 09:46:15</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>1155</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>1002.26</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>1153.14</v>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>1002.26</v>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>2705.5</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>2655.5</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>37719.5</v>
+      </c>
+      <c r="P60" s="2" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>2705.5</v>
+      </c>
+      <c r="R60" s="2" t="n">
+        <v>-1123.5</v>
+      </c>
+      <c r="S60" s="2" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="T60" s="2" t="n">
+        <v>-2.98</v>
+      </c>
+      <c r="U60" s="2" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="V60" s="2" t="n">
+        <v>112336.5</v>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16 09:20:02</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR53900CE</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>1326.95</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16 09:42:31</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>1420</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>1234.06</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>1419.84</v>
+      </c>
+      <c r="J61" s="2" t="n">
+        <v>1234.06</v>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L61" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M61" s="2" t="n">
+        <v>3256.75</v>
+      </c>
+      <c r="N61" s="2" t="n">
+        <v>3206.75</v>
+      </c>
+      <c r="O61" s="2" t="n">
+        <v>46443.25</v>
+      </c>
+      <c r="P61" s="2" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>3256.75</v>
+      </c>
+      <c r="R61" s="2" t="n">
+        <v>-232.75</v>
+      </c>
+      <c r="S61" s="2" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="T61" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="U61" s="2" t="n">
+        <v>21.77</v>
+      </c>
+      <c r="V61" s="2" t="n">
+        <v>115543.25</v>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17 09:20:02</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR54200PE</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>991.15</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17 09:37:03</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>919.6</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>921.77</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>1060.53</v>
+      </c>
+      <c r="J62" s="2" t="n">
+        <v>921.77</v>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L62" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M62" s="2" t="n">
+        <v>-2504.25</v>
+      </c>
+      <c r="N62" s="2" t="n">
+        <v>-2554.25</v>
+      </c>
+      <c r="O62" s="2" t="n">
+        <v>34690.25</v>
+      </c>
+      <c r="P62" s="2" t="n">
+        <v>-7.22</v>
+      </c>
+      <c r="Q62" s="2" t="n">
+        <v>1683.5</v>
+      </c>
+      <c r="R62" s="2" t="n">
+        <v>-2504.25</v>
+      </c>
+      <c r="S62" s="2" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="T62" s="2" t="n">
+        <v>-7.22</v>
+      </c>
+      <c r="U62" s="2" t="n">
+        <v>20.82</v>
+      </c>
+      <c r="V62" s="2" t="n">
+        <v>112989</v>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19 09:20:02</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR53400PE</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>730.15</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19 09:22:25</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>678.55</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>679.04</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>781.26</v>
+      </c>
+      <c r="J63" s="2" t="n">
+        <v>679.04</v>
+      </c>
+      <c r="K63" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L63" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M63" s="2" t="n">
+        <v>-1806</v>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>-1856</v>
+      </c>
+      <c r="O63" s="2" t="n">
+        <v>25555.25</v>
+      </c>
+      <c r="P63" s="2" t="n">
+        <v>-7.07</v>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>637</v>
+      </c>
+      <c r="R63" s="2" t="n">
+        <v>-1806</v>
+      </c>
+      <c r="S63" s="2" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="T63" s="2" t="n">
+        <v>-7.07</v>
+      </c>
+      <c r="U63" s="2" t="n">
+        <v>21.41</v>
+      </c>
+      <c r="V63" s="2" t="n">
+        <v>111133</v>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20 09:20:02</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR54200CE</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>1010.1</v>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20 09:32:53</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>1093.25</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>939.39</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>1080.81</v>
+      </c>
+      <c r="J64" s="2" t="n">
+        <v>939.39</v>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M64" s="2" t="n">
+        <v>2910.25</v>
+      </c>
+      <c r="N64" s="2" t="n">
+        <v>2860.25</v>
+      </c>
+      <c r="O64" s="2" t="n">
+        <v>35353.5</v>
+      </c>
+      <c r="P64" s="2" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="Q64" s="2" t="n">
+        <v>2910.25</v>
+      </c>
+      <c r="R64" s="2" t="n">
+        <v>-2411.5</v>
+      </c>
+      <c r="S64" s="2" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="T64" s="2" t="n">
+        <v>-6.82</v>
+      </c>
+      <c r="U64" s="2" t="n">
+        <v>22.01</v>
+      </c>
+      <c r="V64" s="2" t="n">
+        <v>113993.25</v>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23 09:20:02</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR52100PE</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>979.95</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23 09:50:34</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>1049.1</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>911.35</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>1048.55</v>
+      </c>
+      <c r="J65" s="2" t="n">
+        <v>911.35</v>
+      </c>
+      <c r="K65" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L65" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M65" s="2" t="n">
+        <v>2420.25</v>
+      </c>
+      <c r="N65" s="2" t="n">
+        <v>2370.25</v>
+      </c>
+      <c r="O65" s="2" t="n">
+        <v>34298.25</v>
+      </c>
+      <c r="P65" s="2" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="Q65" s="2" t="n">
+        <v>2420.25</v>
+      </c>
+      <c r="R65" s="2" t="n">
+        <v>227.5</v>
+      </c>
+      <c r="S65" s="2" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="T65" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="U65" s="2" t="n">
+        <v>25.66</v>
+      </c>
+      <c r="V65" s="2" t="n">
+        <v>116363.5</v>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 09:20:02</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR52500CE</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>880.5</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 09:31:22</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>942.4</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>818.86</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>942.14</v>
+      </c>
+      <c r="J66" s="2" t="n">
+        <v>818.86</v>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>2166.5</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>2116.5</v>
+      </c>
+      <c r="O66" s="2" t="n">
+        <v>30817.5</v>
+      </c>
+      <c r="P66" s="2" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="Q66" s="2" t="n">
+        <v>2166.5</v>
+      </c>
+      <c r="R66" s="2" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="S66" s="2" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="T66" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="U66" s="2" t="n">
+        <v>25.06</v>
+      </c>
+      <c r="V66" s="2" t="n">
+        <v>118480</v>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25 09:22:05</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR53500CE</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>748.1</v>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25 09:25:25</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>801</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>695.73</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>800.47</v>
+      </c>
+      <c r="J67" s="2" t="n">
+        <v>695.73</v>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L67" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M67" s="2" t="n">
+        <v>1851.5</v>
+      </c>
+      <c r="N67" s="2" t="n">
+        <v>1801.5</v>
+      </c>
+      <c r="O67" s="2" t="n">
+        <v>26183.5</v>
+      </c>
+      <c r="P67" s="2" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="Q67" s="2" t="n">
+        <v>1851.5</v>
+      </c>
+      <c r="R67" s="2" t="n">
+        <v>-243.25</v>
+      </c>
+      <c r="S67" s="2" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="T67" s="2" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="U67" s="2" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="V67" s="2" t="n">
+        <v>120281.5</v>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-27 09:25:46</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR52800PE</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>593.1</v>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-27 09:30:12</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>644.15</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>551.58</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>634.62</v>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>551.58</v>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>1786.75</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>1736.75</v>
+      </c>
+      <c r="O68" s="2" t="n">
+        <v>20758.5</v>
+      </c>
+      <c r="P68" s="2" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="Q68" s="2" t="n">
+        <v>1786.75</v>
+      </c>
+      <c r="R68" s="2" t="n">
+        <v>-152.25</v>
+      </c>
+      <c r="S68" s="2" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="T68" s="2" t="n">
+        <v>-0.73</v>
+      </c>
+      <c r="U68" s="2" t="n">
+        <v>25.84</v>
+      </c>
+      <c r="V68" s="2" t="n">
+        <v>122018.25</v>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-30 09:20:02</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26MAR51000PE</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>338.1</v>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-30 09:28:20</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>297.45</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>297.53</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>378.67</v>
+      </c>
+      <c r="J69" s="2" t="n">
+        <v>297.53</v>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>-1422.75</v>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>-1472.75</v>
+      </c>
+      <c r="O69" s="2" t="n">
+        <v>11833.5</v>
+      </c>
+      <c r="P69" s="2" t="n">
+        <v>-12.02</v>
+      </c>
+      <c r="Q69" s="2" t="n">
+        <v>411.25</v>
+      </c>
+      <c r="R69" s="2" t="n">
+        <v>-1422.75</v>
+      </c>
+      <c r="S69" s="2" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="T69" s="2" t="n">
+        <v>-12.02</v>
+      </c>
+      <c r="U69" s="2" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="V69" s="2" t="n">
+        <v>120545.5</v>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01 09:20:02</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26APR51400PE</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>1443.9</v>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:25:06</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>1551.3</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>1342.83</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>1544.97</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>1342.83</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>3759</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>3709</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>50536.5</v>
+      </c>
+      <c r="P70" s="2" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="Q70" s="2" t="n">
+        <v>3759</v>
+      </c>
+      <c r="R70" s="2" t="n">
+        <v>-2310</v>
+      </c>
+      <c r="S70" s="2" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="T70" s="2" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="U70" s="2" t="n">
+        <v>25.17</v>
+      </c>
+      <c r="V70" s="2" t="n">
+        <v>124254.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Final compliance and logic fixes: market open wait, holiday/weekend exit, balance cleanup
</commit_message>
<xml_diff>
--- a/logs/Forward Testing Trade History.xlsx
+++ b/logs/Forward Testing Trade History.xlsx
@@ -2,35 +2,192 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23040" windowHeight="8520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -39,12 +196,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -52,9 +395,251 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -65,8 +650,56 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -419,7 +1052,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -429,8 +1061,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V70"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:V73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -444,13 +1076,13 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="14"/>
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -634,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>1.503006012024048</v>
+        <v>1.50300601202405</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
@@ -5948,6 +6580,186 @@
       </c>
       <c r="V70" s="2" t="n">
         <v>124254.5</v>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="n"/>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
+      <c r="M71" s="2" t="n"/>
+      <c r="N71" s="2" t="n"/>
+      <c r="O71" s="2" t="n"/>
+      <c r="P71" s="2" t="n"/>
+      <c r="Q71" s="2" t="n"/>
+      <c r="R71" s="2" t="n"/>
+      <c r="S71" s="2" t="n"/>
+      <c r="T71" s="2" t="n"/>
+      <c r="U71" s="2" t="n"/>
+      <c r="V71" s="2" t="n"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 09:20:02</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26APR51800CE</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>1729.9</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 09:48:41</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>1604.1</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>1608.81</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>1850.99</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>1608.81</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>-4403</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>-4453</v>
+      </c>
+      <c r="O72" s="2" t="n">
+        <v>60546.5</v>
+      </c>
+      <c r="P72" s="2" t="n">
+        <v>-7.27</v>
+      </c>
+      <c r="Q72" s="2" t="n">
+        <v>1750</v>
+      </c>
+      <c r="R72" s="2" t="n">
+        <v>-4403</v>
+      </c>
+      <c r="S72" s="2" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="T72" s="2" t="n">
+        <v>-7.27</v>
+      </c>
+      <c r="U72" s="2" t="n">
+        <v>26.28</v>
+      </c>
+      <c r="V72" s="2" t="n">
+        <v>119751.5</v>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07 09:20:02</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>NSE:BANKNIFTY26APR51900PE</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>1452.6</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07 09:27:27</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>1350.05</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>1350.92</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>1554.28</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>1350.92</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>-3589.25</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>-3639.25</v>
+      </c>
+      <c r="O73" s="2" t="n">
+        <v>50841</v>
+      </c>
+      <c r="P73" s="2" t="n">
+        <v>-7.06</v>
+      </c>
+      <c r="Q73" s="2" t="n">
+        <v>677.25</v>
+      </c>
+      <c r="R73" s="2" t="n">
+        <v>-3589.25</v>
+      </c>
+      <c r="S73" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="T73" s="2" t="n">
+        <v>-7.06</v>
+      </c>
+      <c r="U73" s="2" t="n">
+        <v>25.52</v>
+      </c>
+      <c r="V73" s="2" t="n">
+        <v>116112.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>